<commit_message>
Krama Paatam upgrade and reco
</commit_message>
<xml_diff>
--- a/TS Jatai Ghanam Project/Reconcilation of total vakyams TS.xlsx
+++ b/TS Jatai Ghanam Project/Reconcilation of total vakyams TS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\texts\TS Jatai Ghanam Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B90EEB2-6396-42EA-B034-C68FA68E763D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4DE84D-34F5-4314-BCA6-C5E8EF364496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="62">
   <si>
     <t xml:space="preserve">Reconciliation of Total vAkyams in Krama, Jatai and Ghanam as per Published VedaVMS </t>
   </si>
@@ -217,6 +217,9 @@
   </si>
   <si>
     <t>Grand Total TS</t>
+  </si>
+  <si>
+    <t>Diff</t>
   </si>
 </sst>
 </file>
@@ -265,12 +268,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -285,12 +294,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -578,6 +589,7 @@
     <col min="2" max="2" width="12.5703125" customWidth="1"/>
     <col min="3" max="3" width="16.42578125" customWidth="1"/>
     <col min="4" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="23.25" x14ac:dyDescent="0.35">
@@ -636,7 +648,9 @@
       <c r="E3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="1"/>
+      <c r="F3" s="1" t="s">
+        <v>61</v>
+      </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
@@ -706,12 +720,17 @@
       <c r="B6" s="1">
         <v>1530</v>
       </c>
-      <c r="C6" s="1"/>
+      <c r="C6" s="1">
+        <v>1771</v>
+      </c>
       <c r="D6" s="1">
         <v>1771</v>
       </c>
       <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
+      <c r="F6" s="1">
+        <f>+D6-C6</f>
+        <v>0</v>
+      </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
@@ -732,12 +751,17 @@
       <c r="B7" s="1">
         <v>1690</v>
       </c>
-      <c r="C7" s="1"/>
+      <c r="C7" s="1">
+        <v>1914</v>
+      </c>
       <c r="D7" s="1">
         <v>1914</v>
       </c>
       <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
+      <c r="F7" s="1">
+        <f t="shared" ref="F7:F62" si="0">+D7-C7</f>
+        <v>0</v>
+      </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -758,12 +782,17 @@
       <c r="B8" s="1">
         <v>1567</v>
       </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1">
+      <c r="C8" s="5">
+        <v>1795</v>
+      </c>
+      <c r="D8" s="5">
         <v>1797</v>
       </c>
       <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
+      <c r="F8" s="1">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
@@ -784,12 +813,17 @@
       <c r="B9" s="1">
         <v>1810</v>
       </c>
-      <c r="C9" s="1"/>
+      <c r="C9" s="1">
+        <v>2085</v>
+      </c>
       <c r="D9" s="1">
         <v>2085</v>
       </c>
       <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
+      <c r="F9" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -810,12 +844,17 @@
       <c r="B10" s="1">
         <v>2717</v>
       </c>
-      <c r="C10" s="1"/>
+      <c r="C10" s="1">
+        <v>3087</v>
+      </c>
       <c r="D10" s="1">
         <v>3087</v>
       </c>
       <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
+      <c r="F10" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -836,12 +875,17 @@
       <c r="B11" s="1">
         <v>2509</v>
       </c>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1">
+        <v>2919</v>
+      </c>
       <c r="D11" s="1">
         <v>2919</v>
       </c>
       <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
+      <c r="F11" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -862,12 +906,17 @@
       <c r="B12" s="1">
         <v>2655</v>
       </c>
-      <c r="C12" s="1"/>
+      <c r="C12" s="1">
+        <v>3073</v>
+      </c>
       <c r="D12" s="1">
         <v>3073</v>
       </c>
       <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
+      <c r="F12" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -888,12 +937,17 @@
       <c r="B13" s="1">
         <v>2094</v>
       </c>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1">
+        <v>2450</v>
+      </c>
       <c r="D13" s="1">
         <v>2450</v>
       </c>
       <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
+      <c r="F13" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
@@ -915,13 +969,18 @@
         <f>SUM(B6:B13)</f>
         <v>16572</v>
       </c>
-      <c r="C14" s="1"/>
+      <c r="C14" s="5">
+        <v>19094</v>
+      </c>
       <c r="D14" s="2">
         <f>SUM(D6:D13)</f>
         <v>19096</v>
       </c>
       <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
+      <c r="F14" s="1">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
@@ -961,12 +1020,17 @@
       <c r="B16" s="1">
         <v>3278</v>
       </c>
-      <c r="C16" s="1"/>
+      <c r="C16" s="1">
+        <v>3773</v>
+      </c>
       <c r="D16" s="1">
         <v>3773</v>
       </c>
       <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
+      <c r="F16" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
@@ -987,12 +1051,17 @@
       <c r="B17" s="1">
         <v>3526</v>
       </c>
-      <c r="C17" s="1"/>
+      <c r="C17" s="1">
+        <v>4234</v>
+      </c>
       <c r="D17" s="1">
         <v>4234</v>
       </c>
       <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
+      <c r="F17" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
@@ -1013,12 +1082,17 @@
       <c r="B18" s="1">
         <v>2965</v>
       </c>
-      <c r="C18" s="1"/>
+      <c r="C18" s="1">
+        <v>3384</v>
+      </c>
       <c r="D18" s="1">
         <v>3384</v>
       </c>
       <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
+      <c r="F18" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
@@ -1039,12 +1113,17 @@
       <c r="B19" s="1">
         <v>2406</v>
       </c>
-      <c r="C19" s="1"/>
+      <c r="C19" s="1">
+        <v>2696</v>
+      </c>
       <c r="D19" s="1">
         <v>2696</v>
       </c>
       <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
+      <c r="F19" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
@@ -1065,12 +1144,17 @@
       <c r="B20" s="1">
         <v>3665</v>
       </c>
-      <c r="C20" s="1"/>
+      <c r="C20" s="1">
+        <v>4301</v>
+      </c>
       <c r="D20" s="1">
         <v>4301</v>
       </c>
       <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
+      <c r="F20" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -1091,12 +1175,17 @@
       <c r="B21" s="1">
         <v>3433</v>
       </c>
-      <c r="C21" s="1"/>
+      <c r="C21" s="1">
+        <v>3997</v>
+      </c>
       <c r="D21" s="1">
         <v>3997</v>
       </c>
       <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
+      <c r="F21" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
@@ -1118,13 +1207,19 @@
         <f>SUM(B16:B21)</f>
         <v>19273</v>
       </c>
-      <c r="C22" s="1"/>
+      <c r="C22" s="2">
+        <f>SUM(C16:C21)</f>
+        <v>22385</v>
+      </c>
       <c r="D22" s="2">
         <f>SUM(D16:D21)</f>
         <v>22385</v>
       </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
+      <c r="F22" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
@@ -1164,12 +1259,17 @@
       <c r="B24" s="1">
         <v>2248</v>
       </c>
-      <c r="C24" s="1"/>
+      <c r="C24" s="1">
+        <v>2578</v>
+      </c>
       <c r="D24" s="1">
         <v>2578</v>
       </c>
       <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
+      <c r="F24" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
@@ -1190,12 +1290,17 @@
       <c r="B25" s="1">
         <v>2335</v>
       </c>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1">
+      <c r="C25" s="5">
+        <v>2758</v>
+      </c>
+      <c r="D25" s="5">
         <v>2757</v>
       </c>
       <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
+      <c r="F25" s="1">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
@@ -1216,12 +1321,17 @@
       <c r="B26" s="1">
         <v>1857</v>
       </c>
-      <c r="C26" s="1"/>
+      <c r="C26" s="1">
+        <v>2087</v>
+      </c>
       <c r="D26" s="1">
         <v>2087</v>
       </c>
       <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
+      <c r="F26" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
@@ -1242,12 +1352,17 @@
       <c r="B27" s="1">
         <v>2392</v>
       </c>
-      <c r="C27" s="1"/>
+      <c r="C27" s="1">
+        <v>2760</v>
+      </c>
       <c r="D27" s="1">
         <v>2760</v>
       </c>
       <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
+      <c r="F27" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
@@ -1268,12 +1383,17 @@
       <c r="B28" s="1">
         <v>1790</v>
       </c>
-      <c r="C28" s="1"/>
+      <c r="C28" s="1">
+        <v>2071</v>
+      </c>
       <c r="D28" s="1">
         <v>2071</v>
       </c>
       <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
+      <c r="F28" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
@@ -1295,13 +1415,19 @@
         <f>SUM(B24:B28)</f>
         <v>10622</v>
       </c>
-      <c r="C29" s="1"/>
+      <c r="C29" s="6">
+        <f>SUM(C24:C28)</f>
+        <v>12254</v>
+      </c>
       <c r="D29" s="2">
         <f>SUM(D24:D28)</f>
         <v>12253</v>
       </c>
       <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
+      <c r="F29" s="1">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
@@ -1338,11 +1464,20 @@
       <c r="A31" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
+      <c r="B31" s="1">
+        <v>2293</v>
+      </c>
+      <c r="C31" s="1">
+        <v>2557</v>
+      </c>
+      <c r="D31" s="1">
+        <v>2557</v>
+      </c>
       <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
+      <c r="F31" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
@@ -1360,11 +1495,20 @@
       <c r="A32" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
+      <c r="B32" s="1">
+        <v>2498</v>
+      </c>
+      <c r="C32" s="1">
+        <v>2768</v>
+      </c>
+      <c r="D32" s="1">
+        <v>2768</v>
+      </c>
       <c r="E32" s="1"/>
-      <c r="F32" s="1"/>
+      <c r="F32" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
@@ -1382,11 +1526,20 @@
       <c r="A33" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
+      <c r="B33" s="1">
+        <v>1844</v>
+      </c>
+      <c r="C33" s="1">
+        <v>2195</v>
+      </c>
+      <c r="D33" s="1">
+        <v>2195</v>
+      </c>
       <c r="E33" s="1"/>
-      <c r="F33" s="1"/>
+      <c r="F33" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
@@ -1404,11 +1557,20 @@
       <c r="A34" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1"/>
+      <c r="B34" s="1">
+        <v>1887</v>
+      </c>
+      <c r="C34" s="1">
+        <v>2248</v>
+      </c>
+      <c r="D34" s="1">
+        <v>2248</v>
+      </c>
       <c r="E34" s="1"/>
-      <c r="F34" s="1"/>
+      <c r="F34" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
@@ -1426,11 +1588,20 @@
       <c r="A35" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
+      <c r="B35" s="1">
+        <v>1234</v>
+      </c>
+      <c r="C35" s="1">
+        <v>1417</v>
+      </c>
+      <c r="D35" s="1">
+        <v>1417</v>
+      </c>
       <c r="E35" s="1"/>
-      <c r="F35" s="1"/>
+      <c r="F35" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
@@ -1448,11 +1619,20 @@
       <c r="A36" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="1"/>
+      <c r="B36" s="1">
+        <v>2331</v>
+      </c>
+      <c r="C36" s="1">
+        <v>2676</v>
+      </c>
+      <c r="D36" s="1">
+        <v>2676</v>
+      </c>
       <c r="E36" s="1"/>
-      <c r="F36" s="1"/>
+      <c r="F36" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
@@ -1470,11 +1650,20 @@
       <c r="A37" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B37" s="1"/>
-      <c r="C37" s="1"/>
-      <c r="D37" s="1"/>
+      <c r="B37" s="1">
+        <v>2008</v>
+      </c>
+      <c r="C37" s="1">
+        <v>2210</v>
+      </c>
+      <c r="D37" s="1">
+        <v>2210</v>
+      </c>
       <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
+      <c r="F37" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
@@ -1492,11 +1681,23 @@
       <c r="A38" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
-      <c r="D38" s="1"/>
+      <c r="B38" s="2">
+        <f>SUM(B31:B37)</f>
+        <v>14095</v>
+      </c>
+      <c r="C38" s="2">
+        <f>SUM(C31:C37)</f>
+        <v>16071</v>
+      </c>
+      <c r="D38" s="2">
+        <f>SUM(D31:D37)</f>
+        <v>16071</v>
+      </c>
       <c r="E38" s="1"/>
-      <c r="F38" s="1"/>
+      <c r="F38" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
@@ -1533,11 +1734,20 @@
       <c r="A40" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
+      <c r="B40" s="1">
+        <v>3081</v>
+      </c>
+      <c r="C40" s="1">
+        <v>3544</v>
+      </c>
+      <c r="D40" s="1">
+        <v>3544</v>
+      </c>
       <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
+      <c r="F40" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
@@ -1555,11 +1765,20 @@
       <c r="A41" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
-      <c r="D41" s="1"/>
+      <c r="B41" s="1">
+        <v>3195</v>
+      </c>
+      <c r="C41" s="1">
+        <v>3709</v>
+      </c>
+      <c r="D41" s="1">
+        <v>3709</v>
+      </c>
       <c r="E41" s="1"/>
-      <c r="F41" s="1"/>
+      <c r="F41" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
@@ -1577,11 +1796,20 @@
       <c r="A42" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
+      <c r="B42" s="1">
+        <v>2477</v>
+      </c>
+      <c r="C42" s="5">
+        <v>2959</v>
+      </c>
+      <c r="D42" s="5">
+        <v>2965</v>
+      </c>
       <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
+      <c r="F42" s="1">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
@@ -1599,11 +1827,20 @@
       <c r="A43" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="1"/>
+      <c r="B43" s="1">
+        <v>2906</v>
+      </c>
+      <c r="C43" s="5">
+        <v>3389</v>
+      </c>
+      <c r="D43" s="5">
+        <v>3390</v>
+      </c>
       <c r="E43" s="1"/>
-      <c r="F43" s="1"/>
+      <c r="F43" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
@@ -1621,11 +1858,20 @@
       <c r="A44" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B44" s="1"/>
-      <c r="C44" s="1"/>
-      <c r="D44" s="1"/>
+      <c r="B44" s="1">
+        <v>2727</v>
+      </c>
+      <c r="C44" s="1">
+        <v>3093</v>
+      </c>
+      <c r="D44" s="1">
+        <v>3093</v>
+      </c>
       <c r="E44" s="1"/>
-      <c r="F44" s="1"/>
+      <c r="F44" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
@@ -1643,11 +1889,20 @@
       <c r="A45" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B45" s="1"/>
-      <c r="C45" s="1"/>
-      <c r="D45" s="1"/>
+      <c r="B45" s="1">
+        <v>2436</v>
+      </c>
+      <c r="C45" s="5">
+        <v>2876</v>
+      </c>
+      <c r="D45" s="1">
+        <v>2875</v>
+      </c>
       <c r="E45" s="1"/>
-      <c r="F45" s="1"/>
+      <c r="F45" s="1">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
@@ -1665,11 +1920,20 @@
       <c r="A46" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B46" s="1"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="1"/>
+      <c r="B46" s="1">
+        <v>2582</v>
+      </c>
+      <c r="C46" s="1">
+        <v>2942</v>
+      </c>
+      <c r="D46" s="1">
+        <v>2942</v>
+      </c>
       <c r="E46" s="1"/>
-      <c r="F46" s="1"/>
+      <c r="F46" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
@@ -1687,11 +1951,23 @@
       <c r="A47" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B47" s="1"/>
-      <c r="C47" s="1"/>
-      <c r="D47" s="1"/>
+      <c r="B47" s="2">
+        <f>SUM(B40:B46)</f>
+        <v>19404</v>
+      </c>
+      <c r="C47" s="2">
+        <f>SUM(C40:C46)</f>
+        <v>22512</v>
+      </c>
+      <c r="D47" s="2">
+        <f>SUM(D40:D46)</f>
+        <v>22518</v>
+      </c>
       <c r="E47" s="1"/>
-      <c r="F47" s="1"/>
+      <c r="F47" s="1">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
@@ -1728,11 +2004,20 @@
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B49" s="1"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="1"/>
+      <c r="B49" s="1">
+        <v>3840</v>
+      </c>
+      <c r="C49" s="1">
+        <v>4389</v>
+      </c>
+      <c r="D49" s="1">
+        <v>4389</v>
+      </c>
       <c r="E49" s="1"/>
-      <c r="F49" s="1"/>
+      <c r="F49" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
       <c r="I49" s="1"/>
@@ -1750,11 +2035,20 @@
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B50" s="1"/>
-      <c r="C50" s="1"/>
-      <c r="D50" s="1"/>
+      <c r="B50" s="1">
+        <v>3085</v>
+      </c>
+      <c r="C50" s="1">
+        <v>3628</v>
+      </c>
+      <c r="D50" s="1">
+        <v>3628</v>
+      </c>
       <c r="E50" s="1"/>
-      <c r="F50" s="1"/>
+      <c r="F50" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
@@ -1772,11 +2066,20 @@
       <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="1"/>
+      <c r="B51" s="1">
+        <v>3155</v>
+      </c>
+      <c r="C51" s="1">
+        <v>3675</v>
+      </c>
+      <c r="D51" s="1">
+        <v>3675</v>
+      </c>
       <c r="E51" s="1"/>
-      <c r="F51" s="1"/>
+      <c r="F51" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
@@ -1794,11 +2097,20 @@
       <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B52" s="1"/>
-      <c r="C52" s="1"/>
-      <c r="D52" s="1"/>
+      <c r="B52" s="1">
+        <v>2626</v>
+      </c>
+      <c r="C52" s="1">
+        <v>3036</v>
+      </c>
+      <c r="D52" s="1">
+        <v>3036</v>
+      </c>
       <c r="E52" s="1"/>
-      <c r="F52" s="1"/>
+      <c r="F52" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
       <c r="I52" s="1"/>
@@ -1816,11 +2128,20 @@
       <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B53" s="1"/>
-      <c r="C53" s="1"/>
-      <c r="D53" s="1"/>
+      <c r="B53" s="1">
+        <v>2150</v>
+      </c>
+      <c r="C53" s="1">
+        <v>2514</v>
+      </c>
+      <c r="D53" s="1">
+        <v>2514</v>
+      </c>
       <c r="E53" s="1"/>
-      <c r="F53" s="1"/>
+      <c r="F53" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G53" s="1"/>
       <c r="H53" s="1"/>
       <c r="I53" s="1"/>
@@ -1838,11 +2159,20 @@
       <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B54" s="1"/>
-      <c r="C54" s="1"/>
-      <c r="D54" s="1"/>
+      <c r="B54" s="1">
+        <v>2125</v>
+      </c>
+      <c r="C54" s="1">
+        <v>2473</v>
+      </c>
+      <c r="D54" s="1">
+        <v>2473</v>
+      </c>
       <c r="E54" s="1"/>
-      <c r="F54" s="1"/>
+      <c r="F54" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
       <c r="I54" s="1"/>
@@ -1860,11 +2190,23 @@
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B55" s="1"/>
-      <c r="C55" s="1"/>
-      <c r="D55" s="1"/>
+      <c r="B55" s="2">
+        <f>SUM(B49:B54)</f>
+        <v>16981</v>
+      </c>
+      <c r="C55" s="2">
+        <f>SUM(C49:C54)</f>
+        <v>19715</v>
+      </c>
+      <c r="D55" s="2">
+        <f>SUM(D49:D54)</f>
+        <v>19715</v>
+      </c>
       <c r="E55" s="1"/>
-      <c r="F55" s="1"/>
+      <c r="F55" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
       <c r="I55" s="1"/>
@@ -1901,11 +2243,20 @@
       <c r="A57" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
-      <c r="D57" s="1"/>
+      <c r="B57" s="1">
+        <v>2635</v>
+      </c>
+      <c r="C57" s="5">
+        <v>3089</v>
+      </c>
+      <c r="D57" s="1">
+        <v>3088</v>
+      </c>
       <c r="E57" s="1"/>
-      <c r="F57" s="1"/>
+      <c r="F57" s="1">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
       <c r="I57" s="1"/>
@@ -1923,11 +2274,20 @@
       <c r="A58" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B58" s="1"/>
-      <c r="C58" s="1"/>
-      <c r="D58" s="1"/>
+      <c r="B58" s="1">
+        <v>2330</v>
+      </c>
+      <c r="C58" s="5">
+        <v>2844</v>
+      </c>
+      <c r="D58" s="1">
+        <v>2845</v>
+      </c>
       <c r="E58" s="1"/>
-      <c r="F58" s="1"/>
+      <c r="F58" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
       <c r="I58" s="1"/>
@@ -1945,11 +2305,20 @@
       <c r="A59" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B59" s="1"/>
-      <c r="C59" s="1"/>
-      <c r="D59" s="1"/>
+      <c r="B59" s="1">
+        <v>2123</v>
+      </c>
+      <c r="C59" s="1">
+        <v>2522</v>
+      </c>
+      <c r="D59" s="1">
+        <v>2522</v>
+      </c>
       <c r="E59" s="1"/>
-      <c r="F59" s="1"/>
+      <c r="F59" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G59" s="1"/>
       <c r="H59" s="1"/>
       <c r="I59" s="1"/>
@@ -1967,11 +2336,20 @@
       <c r="A60" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B60" s="1"/>
-      <c r="C60" s="1"/>
-      <c r="D60" s="1"/>
+      <c r="B60" s="1">
+        <v>2621</v>
+      </c>
+      <c r="C60" s="1">
+        <v>3185</v>
+      </c>
+      <c r="D60" s="1">
+        <v>3185</v>
+      </c>
       <c r="E60" s="1"/>
-      <c r="F60" s="1"/>
+      <c r="F60" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G60" s="1"/>
       <c r="H60" s="1"/>
       <c r="I60" s="1"/>
@@ -1989,11 +2367,20 @@
       <c r="A61" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B61" s="1"/>
-      <c r="C61" s="1"/>
-      <c r="D61" s="1"/>
+      <c r="B61" s="1">
+        <v>2631</v>
+      </c>
+      <c r="C61" s="1">
+        <v>3215</v>
+      </c>
+      <c r="D61" s="1">
+        <v>3215</v>
+      </c>
       <c r="E61" s="1"/>
-      <c r="F61" s="1"/>
+      <c r="F61" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G61" s="1"/>
       <c r="H61" s="1"/>
       <c r="I61" s="1"/>
@@ -2008,11 +2395,26 @@
       <c r="R61" s="1"/>
     </row>
     <row r="62" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B62" s="1"/>
-      <c r="C62" s="1"/>
-      <c r="D62" s="1"/>
+      <c r="A62" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B62" s="2">
+        <f>SUM(B57:B61)</f>
+        <v>12340</v>
+      </c>
+      <c r="C62" s="2">
+        <f>SUM(C57:C61)</f>
+        <v>14855</v>
+      </c>
+      <c r="D62" s="2">
+        <f>SUM(D57:D61)</f>
+        <v>14855</v>
+      </c>
       <c r="E62" s="1"/>
-      <c r="F62" s="1"/>
+      <c r="F62" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="G62" s="1"/>
       <c r="H62" s="1"/>
       <c r="I62" s="1"/>
@@ -2027,9 +2429,6 @@
       <c r="R62" s="1"/>
     </row>
     <row r="63" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A63" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
@@ -2071,11 +2470,23 @@
       <c r="A65" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B65" s="1"/>
-      <c r="C65" s="1"/>
-      <c r="D65" s="1"/>
+      <c r="B65" s="2">
+        <f>+B14+B22+B29+B38+B47+B55+B62</f>
+        <v>109287</v>
+      </c>
+      <c r="C65" s="2">
+        <f>+C14+C22+C29+C38+C47+C55+C62</f>
+        <v>126886</v>
+      </c>
+      <c r="D65" s="2">
+        <f>+D14+D22+D29+D38+D47+D55+D62</f>
+        <v>126893</v>
+      </c>
       <c r="E65" s="1"/>
-      <c r="F65" s="1"/>
+      <c r="F65" s="1">
+        <f t="shared" ref="F65" si="1">+D65-C65</f>
+        <v>7</v>
+      </c>
       <c r="G65" s="1"/>
       <c r="H65" s="1"/>
       <c r="I65" s="1"/>
@@ -2814,5 +3225,6 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
TS Vakyam Jatai Kramam reconciliation
</commit_message>
<xml_diff>
--- a/TS Jatai Ghanam Project/Reconcilation of total vakyams TS.xlsx
+++ b/TS Jatai Ghanam Project/Reconcilation of total vakyams TS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\texts\TS Jatai Ghanam Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F23BB5DD-613D-4CD5-A680-42F17E6685DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9BDAC3E-B1D0-4498-9A3B-2732A0A6FE42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -268,18 +268,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -307,8 +301,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -789,10 +783,10 @@
       <c r="B8" s="1">
         <v>1567</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="5">
         <v>1795</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="5">
         <v>1795</v>
       </c>
       <c r="E8" s="1"/>
@@ -976,7 +970,7 @@
         <f>SUM(B6:B13)</f>
         <v>16572</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="5">
         <v>19094</v>
       </c>
       <c r="D14" s="2">
@@ -1297,10 +1291,10 @@
       <c r="B25" s="1">
         <v>2335</v>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="5">
         <v>2757</v>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="5">
         <v>2757</v>
       </c>
       <c r="E25" s="1"/>
@@ -1422,11 +1416,11 @@
         <f>SUM(B24:B28)</f>
         <v>10622</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="6">
         <f>SUM(C24:C28)</f>
         <v>12253</v>
       </c>
-      <c r="D29" s="7">
+      <c r="D29" s="6">
         <f>SUM(D24:D28)</f>
         <v>12253</v>
       </c>
@@ -1806,16 +1800,16 @@
       <c r="B42" s="1">
         <v>2477</v>
       </c>
-      <c r="C42" s="5">
-        <v>2959</v>
-      </c>
-      <c r="D42" s="5">
+      <c r="C42" s="7">
+        <v>2965</v>
+      </c>
+      <c r="D42" s="7">
         <v>2965</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
@@ -1837,16 +1831,16 @@
       <c r="B43" s="1">
         <v>2906</v>
       </c>
-      <c r="C43" s="5">
-        <v>3389</v>
-      </c>
-      <c r="D43" s="5">
+      <c r="C43" s="7">
+        <v>3390</v>
+      </c>
+      <c r="D43" s="7">
         <v>3390</v>
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
@@ -1900,15 +1894,15 @@
         <v>2436</v>
       </c>
       <c r="C45" s="5">
-        <v>2876</v>
-      </c>
-      <c r="D45" s="1">
+        <v>2875</v>
+      </c>
+      <c r="D45" s="5">
         <v>2875</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1">
         <f t="shared" si="0"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
@@ -1964,7 +1958,7 @@
       </c>
       <c r="C47" s="2">
         <f>SUM(C40:C46)</f>
-        <v>22512</v>
+        <v>22518</v>
       </c>
       <c r="D47" s="2">
         <f>SUM(D40:D46)</f>
@@ -1973,7 +1967,7 @@
       <c r="E47" s="1"/>
       <c r="F47" s="1">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
@@ -2254,7 +2248,7 @@
         <v>2635</v>
       </c>
       <c r="C57" s="5">
-        <v>3089</v>
+        <v>3088</v>
       </c>
       <c r="D57" s="1">
         <v>3088</v>
@@ -2262,7 +2256,7 @@
       <c r="E57" s="1"/>
       <c r="F57" s="1">
         <f t="shared" si="0"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
@@ -2285,7 +2279,7 @@
         <v>2330</v>
       </c>
       <c r="C58" s="5">
-        <v>2844</v>
+        <v>2845</v>
       </c>
       <c r="D58" s="1">
         <v>2845</v>
@@ -2293,7 +2287,7 @@
       <c r="E58" s="1"/>
       <c r="F58" s="1">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
@@ -2483,7 +2477,7 @@
       </c>
       <c r="C65" s="2">
         <f>+C14+C22+C29+C38+C47+C55+C62</f>
-        <v>126885</v>
+        <v>126891</v>
       </c>
       <c r="D65" s="2">
         <f>+D14+D22+D29+D38+D47+D55+D62</f>
@@ -2492,7 +2486,7 @@
       <c r="E65" s="1"/>
       <c r="F65" s="1">
         <f t="shared" ref="F65" si="1">+D65-C65</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G65" s="1"/>
       <c r="H65" s="1"/>

</xml_diff>